<commit_message>
Aurigane: squadra uniforme a 3 persone sulle sessioni con il cliente
Recepita la scelta di pianificazione: 3 persone su tutte le sessioni con il
cliente, interviste one-to-one escluse perche' per definizione hanno un solo
intervistatore. Lo scostamento rispetto alle risorse indicate dal contratto e'
segnalato nella colonna Note di ogni fase interessata.

Effetto: front office da 11,91 a 14,53 giornate, margine da -581,75 a
-2.755,75 EUR. Fase 5 e presentazione scendono da 4 a 3 persone, tutte le
altre salgono da 2 a 3.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oZ1NbKKwKBf6GwpJ52mBY
</commit_message>
<xml_diff>
--- a/wbs-aurigane/260909_AURIGANE_WBS_RevOps_Assessment_V.0.9.xlsx
+++ b/wbs-aurigane/260909_AURIGANE_WBS_RevOps_Assessment_V.0.9.xlsx
@@ -1135,7 +1135,7 @@
         <v>1.5</v>
       </c>
       <c r="S3" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T3" s="8" t="n"/>
       <c r="U3" s="11">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="X3" s="6" t="inlineStr">
         <is>
-          <t>2 persone in remoto (Project Manager + RevOps Strategist)</t>
+          <t>3 persone (1 RevOps Strategist Senior + 2 junior) — in remoto</t>
         </is>
       </c>
       <c r="Y3" s="11">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="AB3" s="6" t="inlineStr">
         <is>
-          <t>Offerta § 6.1 — 90 minuti, remoto. L'analisi dati non è un momento erogato: è back office dentro questa fase. La determinazione del perimetro clienti attivi è la voce più incerta del progetto. gg back office: STIMA.</t>
+          <t>Offerta § 6.1 — 90 minuti, remoto. L'analisi dati non è un momento erogato: è back office dentro questa fase. La determinazione del perimetro clienti attivi è la voce più incerta del progetto. gg back office: STIMA. SCOSTAMENTO: il contratto indica 2 risorse su questa fase, il piano ne mette 3 per scelta di pianificazione.</t>
         </is>
       </c>
     </row>
@@ -1253,7 +1253,7 @@
         <v>8</v>
       </c>
       <c r="S4" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T4" s="8" t="n">
         <v>1</v>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="X4" s="6" t="inlineStr">
         <is>
-          <t>2 persone in presenza (RevOps Strategist + CX Specialist) — giornata piena</t>
+          <t>3 persone (1 RevOps Strategist Senior + 2 junior) — in presenza</t>
         </is>
       </c>
       <c r="Y4" s="11">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="AB4" s="6" t="inlineStr">
         <is>
-          <t>Offerta § 6.2 — 8 ore, una giornata di lavoro, in presenza. Tre brand in una sola sessione: è la fase più densa del progetto. gg back office: STIMA.</t>
+          <t>Offerta § 6.2 — 8 ore, una giornata di lavoro, in presenza. Tre brand in una sola sessione: è la fase più densa del progetto. gg back office: STIMA. SCOSTAMENTO: il contratto indica 2 risorse su questa fase, il piano ne mette 3 per scelta di pianificazione.</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
         <v>3</v>
       </c>
       <c r="S5" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T5" s="8" t="n">
         <v>3</v>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="X5" s="6" t="inlineStr">
         <is>
-          <t>2 persone in presenza × 3 sessioni (RevOps Strategist + CX Specialist) — mezze giornate</t>
+          <t>3 persone (1 RevOps Strategist Senior + 2 junior) × 3 sessioni — in presenza</t>
         </is>
       </c>
       <c r="Y5" s="11">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="AB5" s="6" t="inlineStr">
         <is>
-          <t>Offerta § 6.3 — 9 ore complessive: 3 workshop di circa 3 ore, uno per brand, in presenza. Sono le 3 sessioni di mezza giornata che il § 10.1 conta a parte. gg back office: STIMA.</t>
+          <t>Offerta § 6.3 — 9 ore complessive: 3 workshop di circa 3 ore, uno per brand, in presenza. Sono le 3 sessioni di mezza giornata che il § 10.1 conta a parte. gg back office: STIMA. SCOSTAMENTO: il contratto indica 2 risorse su questa fase, il piano ne mette 3 per scelta di pianificazione.</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="X6" s="6" t="inlineStr">
         <is>
-          <t>3 persone in presenza (RevOps Strategist + Process Analyst + UX Researcher)</t>
+          <t>3 persone (1 RevOps Strategist Senior + 2 junior) — in presenza</t>
         </is>
       </c>
       <c r="Y6" s="11">
@@ -1731,7 +1731,7 @@
         <v>2</v>
       </c>
       <c r="S8" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T8" s="8" t="n">
         <v>1</v>
@@ -1749,7 +1749,7 @@
       </c>
       <c r="X8" s="6" t="inlineStr">
         <is>
-          <t>2 persone in presenza (Project Manager + RevOps Strategist) — 3 sessioni in una giornata</t>
+          <t>3 persone (1 RevOps Strategist Senior + 2 junior) × 3 sessioni — in presenza</t>
         </is>
       </c>
       <c r="Y8" s="11">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="AB8" s="6" t="inlineStr">
         <is>
-          <t>Offerta § 6.5 — 3 sessioni da 2 ore nella MEDESIMA giornata: sono 3 incontri e UNA trasferta, ed è così che quadrano le 8 sessioni in presenza del § 10.1. L'Integration Expert del § 9 NON è previsto su questa fase. gg back office: STIMA.</t>
+          <t>Offerta § 6.5 — 3 sessioni da 2 ore nella MEDESIMA giornata: sono 3 incontri e UNA trasferta, ed è così che quadrano le 8 sessioni in presenza del § 10.1. L'Integration Expert del § 9 NON è previsto su questa fase. gg back office: STIMA. SCOSTAMENTO: il contratto indica 2 risorse su questa fase, il piano ne mette 3 per scelta di pianificazione.</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
         <v>3.5</v>
       </c>
       <c r="S9" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T9" s="8" t="n">
         <v>1</v>
@@ -1869,7 +1869,7 @@
       </c>
       <c r="X9" s="6" t="inlineStr">
         <is>
-          <t>4 persone in presenza (RevOps Strategist + CX Specialist + Integration Expert + Project Manager)</t>
+          <t>3 persone (1 RevOps Strategist Senior + 2 junior) — in presenza</t>
         </is>
       </c>
       <c r="Y9" s="11">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="AB9" s="6" t="inlineStr">
         <is>
-          <t>Offerta § 6.6 — 3,5 ore, in presenza, con 4 risorse Impresoft. La roadmap per wave non è una fase: è contenuto del report finale. gg back office: STIMA.</t>
+          <t>Offerta § 6.6 — 3,5 ore, in presenza, con 4 risorse Impresoft. La roadmap per wave non è una fase: è contenuto del report finale. gg back office: STIMA. SCOSTAMENTO: il contratto indica 4 risorse su questa fase, il piano ne mette 3 per scelta di pianificazione.</t>
         </is>
       </c>
     </row>
@@ -2075,7 +2075,7 @@
         <v>2</v>
       </c>
       <c r="S11" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T11" s="8" t="n"/>
       <c r="U11" s="11">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="X11" s="6" t="inlineStr">
         <is>
-          <t>2 persone in remoto (RevOps Strategist + Project Manager)</t>
+          <t>3 persone (1 RevOps Strategist Senior + 2 junior) — in remoto</t>
         </is>
       </c>
       <c r="Y11" s="11">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="AB11" s="6" t="inlineStr">
         <is>
-          <t>FUORI PERIMETRO CONTRATTUALE — l'Offerta non prevede una review fra la Fase 5 e il meeting di presentazione. Aggiunta su richiesta, sul modello del progetto Laica. Durata e squadra sono stime: 2 ore in remoto con 2 persone. gg back office: STIMA.</t>
+          <t>FUORI PERIMETRO CONTRATTUALE — l'Offerta non prevede una review fra la Fase 5 e il meeting di presentazione. Aggiunta su richiesta, sul modello del progetto Laica. Durata e squadra sono stime: 2 ore in remoto con 2 persone. gg back office: STIMA. SCOSTAMENTO: il contratto indica 2 risorse su questa fase, il piano ne mette 3 per scelta di pianificazione.</t>
         </is>
       </c>
     </row>
@@ -2193,7 +2193,7 @@
         <v>2</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T12" s="8" t="n">
         <v>1</v>
@@ -2211,7 +2211,7 @@
       </c>
       <c r="X12" s="6" t="inlineStr">
         <is>
-          <t>4 persone in presenza (RevOps Strategist + CX Specialist + Integration Expert + Project Manager)</t>
+          <t>3 persone (1 RevOps Strategist Senior + 2 junior) — in presenza</t>
         </is>
       </c>
       <c r="Y12" s="11">
@@ -2228,7 +2228,7 @@
       </c>
       <c r="AB12" s="6" t="inlineStr">
         <is>
-          <t>Offerta § 6.6 — 2 ore, in presenza, circa 15 giorni dopo la Fase 5. VINCOLO DI PIANIFICAZIONE. gg back office: STIMA.</t>
+          <t>Offerta § 6.6 — 2 ore, in presenza, circa 15 giorni dopo la Fase 5. VINCOLO DI PIANIFICAZIONE. gg back office: STIMA. SCOSTAMENTO: il contratto indica 4 risorse su questa fase, il piano ne mette 3 per scelta di pianificazione.</t>
         </is>
       </c>
     </row>

</xml_diff>